<commit_message>
Updated KEN model - 2025-12-12 15:17
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_KEN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E57B621-D954-4B49-9245-39A0BB3986D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4471C2BF-9695-4897-89A9-5E2F3E0FB5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="388">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -618,6 +618,9 @@
     <t>wnid offshore potential</t>
   </si>
   <si>
+    <t>ELC_BatIn</t>
+  </si>
+  <si>
     <t>~fi_process</t>
   </si>
   <si>
@@ -1285,6 +1288,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>e_KE15-220,e_w660091166-220</t>
   </si>
 </sst>
 </file>
@@ -3178,7 +3184,7 @@
       </c>
       <c r="L27" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_KE15-220,e_w660091166-220</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -3200,7 +3206,7 @@
       </c>
       <c r="K28" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_KE15-220,e_w660091166-220</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3215,7 +3221,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>19</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -4692,9 +4698,8 @@
     <row r="8" spans="2:25" ht="17.649999999999999">
       <c r="B8" s="20"/>
       <c r="E8" s="26"/>
-      <c r="F8" t="str">
-        <f>C5</f>
-        <v>ELC</v>
+      <c r="F8" t="s">
+        <v>163</v>
       </c>
       <c r="G8" t="str">
         <f>E7</f>
@@ -6017,62 +6022,62 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CFA9138-D956-44BA-B3FF-8D042A900F99}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9662FA59-7D5F-45D1-912C-4FA15601C53A}">
   <dimension ref="B9:M38"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:13">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
-        <v>167</v>
-      </c>
-      <c r="F10" t="s">
-        <v>168</v>
-      </c>
-      <c r="G10" t="s">
-        <v>169</v>
-      </c>
-      <c r="H10" t="s">
-        <v>170</v>
-      </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
       <c r="K10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="L10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="M10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="2:13">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -6081,16 +6086,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L11">
         <v>2.8968976635313326</v>
@@ -6101,13 +6106,13 @@
     </row>
     <row r="12" spans="2:13">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -6116,16 +6121,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L12">
         <v>0.40337662696804566</v>
@@ -6136,13 +6141,13 @@
     </row>
     <row r="13" spans="2:13">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -6151,16 +6156,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L13">
         <v>11.689626123166848</v>
@@ -6171,13 +6176,13 @@
     </row>
     <row r="14" spans="2:13">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -6186,16 +6191,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L14">
         <v>36.16807762931424</v>
@@ -6206,13 +6211,13 @@
     </row>
     <row r="15" spans="2:13">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -6221,16 +6226,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L15">
         <v>12.146792968753148</v>
@@ -6241,13 +6246,13 @@
     </row>
     <row r="16" spans="2:13">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -6256,16 +6261,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K16" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L16">
         <v>7.3042877221233224</v>
@@ -6276,13 +6281,13 @@
     </row>
     <row r="17" spans="2:13">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D17" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -6291,16 +6296,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L17">
         <v>3.9552307996088447</v>
@@ -6311,13 +6316,13 @@
     </row>
     <row r="18" spans="2:13">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -6326,16 +6331,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K18" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L18">
         <v>17.329622089430899</v>
@@ -6346,13 +6351,13 @@
     </row>
     <row r="19" spans="2:13">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -6361,16 +6366,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K19" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="L19">
         <v>11.786576720249853</v>
@@ -6381,13 +6386,13 @@
     </row>
     <row r="20" spans="2:13">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -6396,16 +6401,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K20" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L20">
         <v>9.433500569960966</v>
@@ -6416,13 +6421,13 @@
     </row>
     <row r="21" spans="2:13">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D21" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -6431,16 +6436,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K21" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="L21">
         <v>8.8152849300557854</v>
@@ -6451,13 +6456,13 @@
     </row>
     <row r="22" spans="2:13">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -6466,16 +6471,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K22" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L22">
         <v>14.958068869507889</v>
@@ -6486,13 +6491,13 @@
     </row>
     <row r="23" spans="2:13">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -6501,16 +6506,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K23" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L23">
         <v>11.43145251014559</v>
@@ -6521,13 +6526,13 @@
     </row>
     <row r="24" spans="2:13">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D24" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -6536,16 +6541,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K24" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="L24">
         <v>8.8022630868364313</v>
@@ -6556,13 +6561,13 @@
     </row>
     <row r="25" spans="2:13">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -6571,16 +6576,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K25" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L25">
         <v>25.23431224641401</v>
@@ -6591,13 +6596,13 @@
     </row>
     <row r="26" spans="2:13">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -6606,16 +6611,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K26" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="L26">
         <v>31.037064761761126</v>
@@ -6626,13 +6631,13 @@
     </row>
     <row r="27" spans="2:13">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D27" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -6641,16 +6646,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K27" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="L27">
         <v>3.4722775462637423</v>
@@ -6661,13 +6666,13 @@
     </row>
     <row r="28" spans="2:13">
       <c r="B28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D28" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -6676,16 +6681,16 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K28" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L28">
         <v>22.602581292198185</v>
@@ -6696,13 +6701,13 @@
     </row>
     <row r="29" spans="2:13">
       <c r="B29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D29" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -6711,16 +6716,16 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K29" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L29">
         <v>22.472738272208847</v>
@@ -6731,13 +6736,13 @@
     </row>
     <row r="30" spans="2:13">
       <c r="B30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -6746,16 +6751,16 @@
         <v>21</v>
       </c>
       <c r="G30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K30" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="L30">
         <v>9.86820378976428</v>
@@ -6766,13 +6771,13 @@
     </row>
     <row r="31" spans="2:13">
       <c r="B31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D31" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -6781,16 +6786,16 @@
         <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="K31" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L31">
         <v>8.9861448355695916</v>
@@ -6801,13 +6806,13 @@
     </row>
     <row r="32" spans="2:13">
       <c r="B32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -6816,16 +6821,16 @@
         <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L32">
         <v>24.542131316767524</v>
@@ -6836,13 +6841,13 @@
     </row>
     <row r="33" spans="2:13">
       <c r="B33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -6851,16 +6856,16 @@
         <v>21</v>
       </c>
       <c r="G33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="L33">
         <v>13.40311107600413</v>
@@ -6871,13 +6876,13 @@
     </row>
     <row r="34" spans="2:13">
       <c r="B34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C34" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D34" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -6886,16 +6891,16 @@
         <v>21</v>
       </c>
       <c r="G34" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H34" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J34" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K34" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L34">
         <v>17.135920894226487</v>
@@ -6906,13 +6911,13 @@
     </row>
     <row r="35" spans="2:13">
       <c r="B35" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C35" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D35" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -6921,16 +6926,16 @@
         <v>21</v>
       </c>
       <c r="G35" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H35" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J35" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K35" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L35">
         <v>16.876925927847243</v>
@@ -6941,13 +6946,13 @@
     </row>
     <row r="36" spans="2:13">
       <c r="B36" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C36" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D36" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
@@ -6956,16 +6961,16 @@
         <v>21</v>
       </c>
       <c r="G36" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H36" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J36" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K36" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="L36">
         <v>16.286751959076469</v>
@@ -6976,13 +6981,13 @@
     </row>
     <row r="37" spans="2:13">
       <c r="B37" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C37" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D37" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
@@ -6991,16 +6996,16 @@
         <v>21</v>
       </c>
       <c r="G37" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J37" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K37" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="L37">
         <v>3.0341676299481568</v>
@@ -7011,13 +7016,13 @@
     </row>
     <row r="38" spans="2:13">
       <c r="B38" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C38" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D38" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
@@ -7026,16 +7031,16 @@
         <v>21</v>
       </c>
       <c r="G38" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H38" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J38" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K38" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="L38">
         <v>8.738095228639077</v>
@@ -7050,101 +7055,101 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1319322E-9B94-44A9-85F0-E57F383A607C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25200CC9-D534-4533-B263-1301B7E3B30F}">
   <dimension ref="B9:Z33"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:26">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="W9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="2:26">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
+        <v>166</v>
+      </c>
+      <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
+        <v>166</v>
+      </c>
+      <c r="K10" t="s">
+        <v>232</v>
+      </c>
+      <c r="L10" t="s">
+        <v>233</v>
+      </c>
+      <c r="M10" t="s">
+        <v>234</v>
+      </c>
+      <c r="O10" t="s">
         <v>165</v>
       </c>
-      <c r="D10" t="s">
+      <c r="P10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
+      <c r="Q10" t="s">
         <v>167</v>
       </c>
-      <c r="F10" t="s">
+      <c r="R10" t="s">
         <v>168</v>
       </c>
-      <c r="G10" t="s">
+      <c r="S10" t="s">
         <v>169</v>
       </c>
-      <c r="H10" t="s">
+      <c r="T10" t="s">
         <v>170</v>
       </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
-      <c r="K10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="U10" t="s">
+        <v>171</v>
+      </c>
+      <c r="W10" t="s">
+        <v>166</v>
+      </c>
+      <c r="X10" t="s">
         <v>232</v>
       </c>
-      <c r="M10" t="s">
+      <c r="Y10" t="s">
         <v>233</v>
       </c>
-      <c r="O10" t="s">
-        <v>164</v>
-      </c>
-      <c r="P10" t="s">
-        <v>165</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>166</v>
-      </c>
-      <c r="R10" t="s">
-        <v>167</v>
-      </c>
-      <c r="S10" t="s">
-        <v>168</v>
-      </c>
-      <c r="T10" t="s">
-        <v>169</v>
-      </c>
-      <c r="U10" t="s">
-        <v>170</v>
-      </c>
-      <c r="W10" t="s">
-        <v>165</v>
-      </c>
-      <c r="X10" t="s">
-        <v>231</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>232</v>
-      </c>
       <c r="Z10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="2:26">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -7153,16 +7158,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="L11">
         <v>2.3509656412756068</v>
@@ -7171,13 +7176,13 @@
         <v>0.109836021041595</v>
       </c>
       <c r="O11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="Q11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="R11" t="s">
         <v>10</v>
@@ -7186,16 +7191,16 @@
         <v>21</v>
       </c>
       <c r="T11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="X11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Y11">
         <v>8.3782499999999995</v>
@@ -7206,13 +7211,13 @@
     </row>
     <row r="12" spans="2:26">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D12" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -7221,16 +7226,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K12" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L12">
         <v>8.646252729661045</v>
@@ -7239,13 +7244,13 @@
         <v>0.2149080559560089</v>
       </c>
       <c r="O12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Q12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="R12" t="s">
         <v>10</v>
@@ -7254,16 +7259,16 @@
         <v>21</v>
       </c>
       <c r="T12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="X12" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="Y12">
         <v>8.2312499999999993</v>
@@ -7274,13 +7279,13 @@
     </row>
     <row r="13" spans="2:26">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -7289,16 +7294,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="L13">
         <v>1.5817501567892978</v>
@@ -7307,13 +7312,13 @@
         <v>0.33309194745150211</v>
       </c>
       <c r="O13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Q13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="R13" t="s">
         <v>10</v>
@@ -7322,16 +7327,16 @@
         <v>21</v>
       </c>
       <c r="T13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="X13" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="Y13">
         <v>8.9497499999999999</v>
@@ -7342,13 +7347,13 @@
     </row>
     <row r="14" spans="2:26">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D14" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -7357,16 +7362,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L14">
         <v>25.065653532979095</v>
@@ -7375,13 +7380,13 @@
         <v>0.2502810608198982</v>
       </c>
       <c r="O14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="Q14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="R14" t="s">
         <v>10</v>
@@ -7390,16 +7395,16 @@
         <v>21</v>
       </c>
       <c r="T14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="X14" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="Y14">
         <v>0.47775000000000001</v>
@@ -7410,13 +7415,13 @@
     </row>
     <row r="15" spans="2:26">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D15" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -7425,16 +7430,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K15" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L15">
         <v>5.9815028333306417</v>
@@ -7443,13 +7448,13 @@
         <v>0.2858632512923428</v>
       </c>
       <c r="O15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="Q15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="R15" t="s">
         <v>10</v>
@@ -7458,16 +7463,16 @@
         <v>21</v>
       </c>
       <c r="T15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="X15" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="Y15">
         <v>0.13425000000000001</v>
@@ -7478,13 +7483,13 @@
     </row>
     <row r="16" spans="2:26">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D16" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -7493,16 +7498,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K16" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="L16">
         <v>12.399137262716737</v>
@@ -7511,13 +7516,13 @@
         <v>0.34572608805755811</v>
       </c>
       <c r="O16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P16" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Q16" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="R16" t="s">
         <v>10</v>
@@ -7526,16 +7531,16 @@
         <v>21</v>
       </c>
       <c r="T16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W16" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="X16" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Y16">
         <v>3.92625</v>
@@ -7546,13 +7551,13 @@
     </row>
     <row r="17" spans="2:26">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -7561,16 +7566,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="L17">
         <v>20.79964040594967</v>
@@ -7579,13 +7584,13 @@
         <v>0.395906817887822</v>
       </c>
       <c r="O17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P17" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="R17" t="s">
         <v>10</v>
@@ -7594,16 +7599,16 @@
         <v>21</v>
       </c>
       <c r="T17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W17" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="X17" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="Y17">
         <v>2.2530000000000001</v>
@@ -7614,13 +7619,13 @@
     </row>
     <row r="18" spans="2:26">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D18" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -7629,16 +7634,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="L18">
         <v>9.3777415849931209</v>
@@ -7647,13 +7652,13 @@
         <v>0.33056297534614321</v>
       </c>
       <c r="O18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Q18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="R18" t="s">
         <v>10</v>
@@ -7662,16 +7667,16 @@
         <v>21</v>
       </c>
       <c r="T18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="X18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Y18">
         <v>6.1852499999999999</v>
@@ -7682,13 +7687,13 @@
     </row>
     <row r="19" spans="2:26">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D19" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -7697,16 +7702,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K19" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="L19">
         <v>26.805551801109274</v>
@@ -7715,13 +7720,13 @@
         <v>0.27452187627990171</v>
       </c>
       <c r="O19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P19" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="Q19" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="R19" t="s">
         <v>10</v>
@@ -7730,16 +7735,16 @@
         <v>21</v>
       </c>
       <c r="T19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W19" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="X19" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Y19">
         <v>10.093500000000001</v>
@@ -7750,13 +7755,13 @@
     </row>
     <row r="20" spans="2:26">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D20" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -7765,16 +7770,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K20" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="L20">
         <v>20.571034962175187</v>
@@ -7783,13 +7788,13 @@
         <v>0.31186545842804159</v>
       </c>
       <c r="O20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="Q20" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="R20" t="s">
         <v>10</v>
@@ -7798,16 +7803,16 @@
         <v>21</v>
       </c>
       <c r="T20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="X20" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Y20">
         <v>6.7417499999999997</v>
@@ -7818,13 +7823,13 @@
     </row>
     <row r="21" spans="2:26">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D21" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -7833,16 +7838,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K21" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="L21">
         <v>15.316017274089829</v>
@@ -7853,13 +7858,13 @@
     </row>
     <row r="22" spans="2:26">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D22" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -7868,16 +7873,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K22" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="L22">
         <v>2.3755122289527617</v>
@@ -7888,13 +7893,13 @@
     </row>
     <row r="23" spans="2:26">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D23" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -7903,16 +7908,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K23" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="L23">
         <v>15.32235174795542</v>
@@ -7923,13 +7928,13 @@
     </row>
     <row r="24" spans="2:26">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D24" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -7938,16 +7943,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K24" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L24">
         <v>4.3876485804695786</v>
@@ -7958,13 +7963,13 @@
     </row>
     <row r="25" spans="2:26">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D25" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -7973,16 +7978,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K25" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L25">
         <v>6.1536321015103308</v>
@@ -7993,13 +7998,13 @@
     </row>
     <row r="26" spans="2:26">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D26" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -8008,16 +8013,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K26" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="L26">
         <v>3.7458169954306517</v>
@@ -8028,13 +8033,13 @@
     </row>
     <row r="27" spans="2:26">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D27" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -8043,16 +8048,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K27" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="L27">
         <v>2.899127302163282</v>
@@ -8063,13 +8068,13 @@
     </row>
     <row r="28" spans="2:26">
       <c r="B28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D28" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -8078,16 +8083,16 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J28" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K28" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L28">
         <v>0.58029073588183855</v>
@@ -8098,13 +8103,13 @@
     </row>
     <row r="29" spans="2:26">
       <c r="B29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D29" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -8113,16 +8118,16 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J29" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K29" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="L29">
         <v>1.000771006718568</v>
@@ -8133,13 +8138,13 @@
     </row>
     <row r="30" spans="2:26">
       <c r="B30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D30" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -8148,16 +8153,16 @@
         <v>21</v>
       </c>
       <c r="G30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J30" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K30" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="L30">
         <v>2.8972001484003882</v>
@@ -8168,13 +8173,13 @@
     </row>
     <row r="31" spans="2:26">
       <c r="B31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -8183,16 +8188,16 @@
         <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K31" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="L31">
         <v>3.577895438171812</v>
@@ -8203,13 +8208,13 @@
     </row>
     <row r="32" spans="2:26">
       <c r="B32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C32" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D32" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -8218,16 +8223,16 @@
         <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J32" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K32" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L32">
         <v>0.91282903432358287</v>
@@ -8238,13 +8243,13 @@
     </row>
     <row r="33" spans="2:13">
       <c r="B33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C33" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D33" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -8253,16 +8258,16 @@
         <v>21</v>
       </c>
       <c r="G33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J33" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K33" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="L33">
         <v>1.8165822236221094</v>
@@ -8277,27 +8282,27 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D095291-EB73-4E24-BCA5-59E5EB4B7EDA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48D6FBDE-C7A5-4038-9CD6-F890633CB145}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:16">
       <c r="B9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="2:16">
       <c r="B10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E10">
         <v>2023</v>
@@ -8312,30 +8317,30 @@
         <v>54</v>
       </c>
       <c r="J10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="2:16">
       <c r="B11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
@@ -8356,10 +8361,10 @@
         <v>146</v>
       </c>
       <c r="J11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="M11" t="s">
         <v>10</v>
@@ -8368,15 +8373,15 @@
         <v>21</v>
       </c>
       <c r="O11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="12" spans="2:16">
       <c r="B12" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
@@ -8394,13 +8399,13 @@
         <v>0.5</v>
       </c>
       <c r="H12" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="M12" t="s">
         <v>10</v>
@@ -8409,15 +8414,15 @@
         <v>21</v>
       </c>
       <c r="O12" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P12" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="13" spans="2:16">
       <c r="B13" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C13" t="s">
         <v>31</v>
@@ -8435,13 +8440,13 @@
         <v>4400</v>
       </c>
       <c r="H13" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K13" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="M13" t="s">
         <v>10</v>
@@ -8450,15 +8455,15 @@
         <v>21</v>
       </c>
       <c r="O13" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P13" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="14" spans="2:16">
       <c r="B14" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
@@ -8476,13 +8481,13 @@
         <v>155</v>
       </c>
       <c r="H14" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="M14" t="s">
         <v>10</v>
@@ -8491,15 +8496,15 @@
         <v>21</v>
       </c>
       <c r="O14" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P14" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="2:16">
       <c r="B15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -8517,13 +8522,13 @@
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="J15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="M15" t="s">
         <v>10</v>
@@ -8532,15 +8537,15 @@
         <v>21</v>
       </c>
       <c r="O15" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P15" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="16" spans="2:16">
       <c r="B16" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
@@ -8561,10 +8566,10 @@
         <v>146</v>
       </c>
       <c r="J16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K16" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="M16" t="s">
         <v>10</v>
@@ -8573,15 +8578,15 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P16" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="17" spans="2:16">
       <c r="B17" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
@@ -8599,13 +8604,13 @@
         <v>0.5</v>
       </c>
       <c r="H17" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K17" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="M17" t="s">
         <v>10</v>
@@ -8614,15 +8619,15 @@
         <v>21</v>
       </c>
       <c r="O17" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P17" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="18" spans="2:16">
       <c r="B18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C18" t="s">
         <v>31</v>
@@ -8640,13 +8645,13 @@
         <v>2050</v>
       </c>
       <c r="H18" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K18" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="M18" t="s">
         <v>10</v>
@@ -8655,15 +8660,15 @@
         <v>21</v>
       </c>
       <c r="O18" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P18" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="19" spans="2:16">
       <c r="B19" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
@@ -8681,13 +8686,13 @@
         <v>70</v>
       </c>
       <c r="H19" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K19" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="M19" t="s">
         <v>10</v>
@@ -8696,15 +8701,15 @@
         <v>21</v>
       </c>
       <c r="O19" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P19" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="20" spans="2:16">
       <c r="B20" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C20" t="s">
         <v>31</v>
@@ -8722,13 +8727,13 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="J20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K20" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M20" t="s">
         <v>10</v>
@@ -8737,15 +8742,15 @@
         <v>21</v>
       </c>
       <c r="O20" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P20" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="21" spans="2:16">
       <c r="B21" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C21" t="s">
         <v>33</v>
@@ -8766,10 +8771,10 @@
         <v>146</v>
       </c>
       <c r="J21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K21" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M21" t="s">
         <v>10</v>
@@ -8778,15 +8783,15 @@
         <v>21</v>
       </c>
       <c r="O21" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P21" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="22" spans="2:16">
       <c r="B22" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C22" t="s">
         <v>33</v>
@@ -8804,13 +8809,13 @@
         <v>700</v>
       </c>
       <c r="H22" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K22" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="M22" t="s">
         <v>10</v>
@@ -8819,15 +8824,15 @@
         <v>21</v>
       </c>
       <c r="O22" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P22" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C23" t="s">
         <v>33</v>
@@ -8845,13 +8850,13 @@
         <v>25</v>
       </c>
       <c r="H23" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K23" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="M23" t="s">
         <v>10</v>
@@ -8860,15 +8865,15 @@
         <v>21</v>
       </c>
       <c r="O23" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P23" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="24" spans="2:16">
       <c r="B24" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C24" t="s">
         <v>33</v>
@@ -8889,10 +8894,10 @@
         <v>146</v>
       </c>
       <c r="J24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K24" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="M24" t="s">
         <v>10</v>
@@ -8901,15 +8906,15 @@
         <v>21</v>
       </c>
       <c r="O24" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P24" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="25" spans="2:16">
       <c r="B25" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C25" t="s">
         <v>33</v>
@@ -8927,13 +8932,13 @@
         <v>1850</v>
       </c>
       <c r="H25" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K25" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M25" t="s">
         <v>10</v>
@@ -8942,15 +8947,15 @@
         <v>21</v>
       </c>
       <c r="O25" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P25" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="26" spans="2:16">
       <c r="B26" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C26" t="s">
         <v>33</v>
@@ -8968,13 +8973,13 @@
         <v>65</v>
       </c>
       <c r="H26" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K26" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M26" t="s">
         <v>10</v>
@@ -8983,15 +8988,15 @@
         <v>21</v>
       </c>
       <c r="O26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P26" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="27" spans="2:16">
       <c r="B27" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C27" t="s">
         <v>32</v>
@@ -9012,10 +9017,10 @@
         <v>146</v>
       </c>
       <c r="J27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K27" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="M27" t="s">
         <v>10</v>
@@ -9024,15 +9029,15 @@
         <v>21</v>
       </c>
       <c r="O27" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P27" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="28" spans="2:16">
       <c r="B28" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C28" t="s">
         <v>32</v>
@@ -9050,12 +9055,12 @@
         <v>3550</v>
       </c>
       <c r="H28" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="B29" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C29" t="s">
         <v>32</v>
@@ -9073,12 +9078,12 @@
         <v>135</v>
       </c>
       <c r="H29" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="30" spans="2:16">
       <c r="B30" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C30" t="s">
         <v>33</v>
@@ -9101,7 +9106,7 @@
     </row>
     <row r="31" spans="2:16">
       <c r="B31" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C31" t="s">
         <v>33</v>
@@ -9119,12 +9124,12 @@
         <v>400</v>
       </c>
       <c r="H31" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="32" spans="2:16">
       <c r="B32" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C32" t="s">
         <v>33</v>
@@ -9142,12 +9147,12 @@
         <v>20</v>
       </c>
       <c r="H32" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="33" spans="2:8">
       <c r="B33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C33" t="s">
         <v>28</v>
@@ -9170,7 +9175,7 @@
     </row>
     <row r="34" spans="2:8">
       <c r="B34" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C34" t="s">
         <v>28</v>
@@ -9188,12 +9193,12 @@
         <v>0.5</v>
       </c>
       <c r="H34" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="35" spans="2:8">
       <c r="B35" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
@@ -9211,12 +9216,12 @@
         <v>2100</v>
       </c>
       <c r="H35" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="36" spans="2:8">
       <c r="B36" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
@@ -9234,12 +9239,12 @@
         <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="37" spans="2:8">
       <c r="B37" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
@@ -9257,12 +9262,12 @@
         <v>4</v>
       </c>
       <c r="H37" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="38" spans="2:8">
       <c r="B38" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C38" t="s">
         <v>33</v>
@@ -9285,7 +9290,7 @@
     </row>
     <row r="39" spans="2:8">
       <c r="B39" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -9303,12 +9308,12 @@
         <v>2100</v>
       </c>
       <c r="H39" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="40" spans="2:8">
       <c r="B40" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C40" t="s">
         <v>33</v>
@@ -9326,12 +9331,12 @@
         <v>85</v>
       </c>
       <c r="H40" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="41" spans="2:8">
       <c r="B41" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
@@ -9354,7 +9359,7 @@
     </row>
     <row r="42" spans="2:8">
       <c r="B42" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C42" t="s">
         <v>32</v>
@@ -9372,12 +9377,12 @@
         <v>4200</v>
       </c>
       <c r="H42" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="43" spans="2:8">
       <c r="B43" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C43" t="s">
         <v>32</v>
@@ -9395,12 +9400,12 @@
         <v>190</v>
       </c>
       <c r="H43" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="44" spans="2:8">
       <c r="B44" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C44" t="s">
         <v>36</v>
@@ -9423,7 +9428,7 @@
     </row>
     <row r="45" spans="2:8">
       <c r="B45" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C45" t="s">
         <v>36</v>
@@ -9441,12 +9446,12 @@
         <v>4000</v>
       </c>
       <c r="H45" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="46" spans="2:8">
       <c r="B46" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C46" t="s">
         <v>36</v>
@@ -9464,12 +9469,12 @@
         <v>170</v>
       </c>
       <c r="H46" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="47" spans="2:8">
       <c r="B47" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C47" t="s">
         <v>32</v>
@@ -9492,7 +9497,7 @@
     </row>
     <row r="48" spans="2:8">
       <c r="B48" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C48" t="s">
         <v>32</v>
@@ -9510,12 +9515,12 @@
         <v>4300</v>
       </c>
       <c r="H48" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="49" spans="2:8">
       <c r="B49" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C49" t="s">
         <v>32</v>
@@ -9533,12 +9538,12 @@
         <v>165</v>
       </c>
       <c r="H49" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="50" spans="2:8">
       <c r="B50" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C50" t="s">
         <v>27</v>
@@ -9561,7 +9566,7 @@
     </row>
     <row r="51" spans="2:8">
       <c r="B51" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C51" t="s">
         <v>27</v>
@@ -9579,12 +9584,12 @@
         <v>0.23</v>
       </c>
       <c r="H51" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="52" spans="2:8">
       <c r="B52" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C52" t="s">
         <v>27</v>
@@ -9602,12 +9607,12 @@
         <v>550</v>
       </c>
       <c r="H52" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="53" spans="2:8">
       <c r="B53" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C53" t="s">
         <v>27</v>
@@ -9625,12 +9630,12 @@
         <v>18</v>
       </c>
       <c r="H53" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="54" spans="2:8">
       <c r="B54" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C54" t="s">
         <v>27</v>
@@ -9648,12 +9653,12 @@
         <v>1.5</v>
       </c>
       <c r="H54" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="55" spans="2:8">
       <c r="B55" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C55" t="s">
         <v>32</v>
@@ -9676,7 +9681,7 @@
     </row>
     <row r="56" spans="2:8">
       <c r="B56" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C56" t="s">
         <v>32</v>
@@ -9694,12 +9699,12 @@
         <v>1300</v>
       </c>
       <c r="H56" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="57" spans="2:8">
       <c r="B57" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C57" t="s">
         <v>32</v>
@@ -9717,12 +9722,12 @@
         <v>45</v>
       </c>
       <c r="H57" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="58" spans="2:8">
       <c r="B58" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C58" t="s">
         <v>32</v>
@@ -9745,7 +9750,7 @@
     </row>
     <row r="59" spans="2:8">
       <c r="B59" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C59" t="s">
         <v>32</v>
@@ -9763,12 +9768,12 @@
         <v>1600</v>
       </c>
       <c r="H59" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="60" spans="2:8">
       <c r="B60" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C60" t="s">
         <v>32</v>
@@ -9786,12 +9791,12 @@
         <v>55</v>
       </c>
       <c r="H60" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="61" spans="2:8">
       <c r="B61" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C61" t="s">
         <v>32</v>
@@ -9814,7 +9819,7 @@
     </row>
     <row r="62" spans="2:8">
       <c r="B62" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C62" t="s">
         <v>32</v>
@@ -9832,12 +9837,12 @@
         <v>1900</v>
       </c>
       <c r="H62" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="63" spans="2:8">
       <c r="B63" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
@@ -9855,15 +9860,15 @@
         <v>70</v>
       </c>
       <c r="H63" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="64" spans="2:8">
       <c r="B64" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C64" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D64" t="s">
         <v>19</v>
@@ -9883,10 +9888,10 @@
     </row>
     <row r="65" spans="2:8">
       <c r="B65" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C65" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D65" t="s">
         <v>19</v>
@@ -9901,15 +9906,15 @@
         <v>0.43</v>
       </c>
       <c r="H65" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="66" spans="2:8">
       <c r="B66" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C66" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D66" t="s">
         <v>19</v>
@@ -9924,15 +9929,15 @@
         <v>2200</v>
       </c>
       <c r="H66" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="67" spans="2:8">
       <c r="B67" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C67" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D67" t="s">
         <v>19</v>
@@ -9947,15 +9952,15 @@
         <v>65</v>
       </c>
       <c r="H67" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="B68" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C68" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D68" t="s">
         <v>19</v>
@@ -9970,15 +9975,15 @@
         <v>3</v>
       </c>
       <c r="H68" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="69" spans="2:8">
       <c r="B69" t="s">
+        <v>384</v>
+      </c>
+      <c r="C69" t="s">
         <v>383</v>
-      </c>
-      <c r="C69" t="s">
-        <v>382</v>
       </c>
       <c r="D69" t="s">
         <v>19</v>
@@ -9998,10 +10003,10 @@
     </row>
     <row r="70" spans="2:8">
       <c r="B70" t="s">
+        <v>384</v>
+      </c>
+      <c r="C70" t="s">
         <v>383</v>
-      </c>
-      <c r="C70" t="s">
-        <v>382</v>
       </c>
       <c r="D70" t="s">
         <v>19</v>
@@ -10016,15 +10021,15 @@
         <v>0.35000000000000003</v>
       </c>
       <c r="H70" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="71" spans="2:8">
       <c r="B71" t="s">
+        <v>384</v>
+      </c>
+      <c r="C71" t="s">
         <v>383</v>
-      </c>
-      <c r="C71" t="s">
-        <v>382</v>
       </c>
       <c r="D71" t="s">
         <v>19</v>
@@ -10039,15 +10044,15 @@
         <v>1470</v>
       </c>
       <c r="H71" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="72" spans="2:8">
       <c r="B72" t="s">
+        <v>384</v>
+      </c>
+      <c r="C72" t="s">
         <v>383</v>
-      </c>
-      <c r="C72" t="s">
-        <v>382</v>
       </c>
       <c r="D72" t="s">
         <v>19</v>
@@ -10062,15 +10067,15 @@
         <v>38</v>
       </c>
       <c r="H72" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="73" spans="2:8">
       <c r="B73" t="s">
+        <v>384</v>
+      </c>
+      <c r="C73" t="s">
         <v>383</v>
-      </c>
-      <c r="C73" t="s">
-        <v>382</v>
       </c>
       <c r="D73" t="s">
         <v>19</v>
@@ -10085,7 +10090,7 @@
         <v>1.5</v>
       </c>
       <c r="H73" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>